<commit_message>
Expand Coventry / Warwick block in November digest
Add Bill Bailey (CBS Arena, 13 Nov), The Feeling (hmv Empire, 26 Nov) and
Melanie C (hmv Empire, 28 Nov); the block now has five events.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_11.1-11.30.xlsx
+++ b/data/UK_Events_TrackB_11.1-11.30.xlsx
@@ -13,7 +13,7 @@
     <sheet name="待核实与缺口" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Track B 30天活动'!$A$1:$O$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Track B 30天活动'!$A$1:$O$126</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'汇总'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'社群覆盖清单'!$A$1:$E$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核实与缺口'!$A$1:$B$12</definedName>
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O123"/>
+  <dimension ref="A1:O126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6257,7 +6257,10 @@
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: COVENTRY &amp; WARWICK 👇
 🎲 EPIC.LAN TT11 Tabletop Weekender, Coventry — a weekend of board games plus a mini LAN, 20–22 Nov.
-🎤 Comedy at Warwick Arts Centre, University of Warwick — Nish Kumar, Flo &amp; Joan, Jonathan Pie &amp; more, 12–27 Nov.</t>
+🎤 Comedy at Warwick Arts Centre, University of Warwick — Nish Kumar, Flo &amp; Joan, Jonathan Pie &amp; more, 12–27 Nov.
+🎸 The Feeling, hmv Empire, Coventry — 20 years of "Twelve Stops and Home", 26 Nov.
+🎤 Bill Bailey, Coventry Building Society Arena — a big Friday night of comedy, 13 Nov.
+🎤 Melanie C (intimate show), hmv Empire, Coventry — a Spice Girl up close (check tickets), 28 Nov.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -6387,32 +6390,17 @@
       </c>
     </row>
     <row r="84" ht="58" customHeight="1">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>University of Leicester / De Montfort University</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>待制作：University of Leicester.png</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>🔍 Event Radar (UK) — what's worth doing this month.
-This month: LEICESTER 👇
-📝 John Cooper Clarke, De Montfort Hall, Leicester — the punk poet live, 25 Nov.
-🎄 Leicester Christmas Market &amp; ice rink, Gallowtree Gate — festive stalls &amp; skating (dates TBC), mid-Nov.</t>
-        </is>
-      </c>
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="4" t="n"/>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>John Cooper Clarke 巡演 莱斯特站</t>
+          <t>The Feeling《Twelve Stops and Home》20 周年巡演</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>De Montfort Hall, Granville Road, Leicester LE1 7RU</t>
+          <t>hmv Empire, Hales Street, Coventry CV1 1JD</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -6422,12 +6410,12 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>25 Nov 2026（周三）</t>
+          <t>26 Nov 2026（周四）19:00</t>
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>年轻人娱乐(诗歌/Live)</t>
+          <t>年轻人娱乐(Live Music/英伦流行)</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -6437,17 +6425,17 @@
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>多个票务汇总站（Songkick、Stereoboard 等）日期一致；朋克诗人，现场口碑好</t>
+          <t>JamBase 等多个票务站日期一致；成名专辑 20 周年巡演</t>
         </is>
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/venues/1771-de-montfort-hall/calendar ; https://www.stereoboard.com/venues/leicester/de-montfort-hall</t>
+          <t>https://www.jambase.com/show/the-feeling-hmv-empire-coventry-20261126 ; https://www.hmvempire.com/</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
         <is>
-          <t>英国标志性朋克诗人；De Montfort Hall 离 DMU、Leicester 大学都近</t>
+          <t>票价约 £38.50 起；场馆在市中心，Coventry 大学走路就到</t>
         </is>
       </c>
       <c r="M84" s="5" t="inlineStr">
@@ -6472,77 +6460,287 @@
       <c r="C85" s="4" t="n"/>
       <c r="D85" s="2" t="inlineStr">
         <is>
+          <t>Bill Bailey 单口喜剧巡演 考文垂站</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Coventry Building Society Arena, Judds Lane, Coventry CV6 6GE</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>13 Nov 2026（周五）20:00</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(喜剧)</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>Ticketmaster 正规售票；英国顶级喜剧人，体育馆级别的场次</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.co.uk/coventry-building-society-arena-tickets-coventry/venue/452099 ; https://www.coventrybuildingsocietyarena.co.uk/</t>
+        </is>
+      </c>
+      <c r="L85" s="5" t="inlineStr">
+        <is>
+          <t>周五晚上的大场喜剧；体育馆在城北，有火车站（Coventry Arena）</t>
+        </is>
+      </c>
+      <c r="M85" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N85" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O85" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="58" customHeight="1">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="4" t="n"/>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Melanie C 小型专场</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>hmv Empire, Hales Street, Coventry CV1 1JD</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>28 Nov 2026（周六）</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/流行)</t>
+        </is>
+      </c>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>只在场馆官网日程里看到，没有第三方票务确认</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hmvempire.com/</t>
+        </is>
+      </c>
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>前辣妹组合成员的近距离小场；推之前确认一下票务页</t>
+        </is>
+      </c>
+      <c r="M86" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O86" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="58" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>University of Leicester / De Montfort University</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>待制作：University of Leicester.png</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>🔍 Event Radar (UK) — what's worth doing this month.
+This month: LEICESTER 👇
+📝 John Cooper Clarke, De Montfort Hall, Leicester — the punk poet live, 25 Nov.
+🎄 Leicester Christmas Market &amp; ice rink, Gallowtree Gate — festive stalls &amp; skating (dates TBC), mid-Nov.</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>John Cooper Clarke 巡演 莱斯特站</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>De Montfort Hall, Granville Road, Leicester LE1 7RU</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>25 Nov 2026（周三）</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(诗歌/Live)</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>多个票务汇总站（Songkick、Stereoboard 等）日期一致；朋克诗人，现场口碑好</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr">
+        <is>
+          <t>https://www.songkick.com/venues/1771-de-montfort-hall/calendar ; https://www.stereoboard.com/venues/leicester/de-montfort-hall</t>
+        </is>
+      </c>
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>英国标志性朋克诗人；De Montfort Hall 离 DMU、Leicester 大学都近</t>
+        </is>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N87" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O87" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="58" customHeight="1">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="4" t="n"/>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
           <t>Leicester Christmas Market &amp; 溜冰场</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>Gallowtree Gate 一带, Leicester city centre</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G85" s="5" t="inlineStr">
+      <c r="G88" s="5" t="inlineStr">
         <is>
           <t>⚠️12 Nov – 27 Dec 2026（官网写这个日期，但页面还留着 2024 年的文字，待核实）</t>
         </is>
       </c>
-      <c r="H85" s="5" t="inlineStr">
+      <c r="H88" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市/滑冰)</t>
         </is>
       </c>
-      <c r="I85" s="7" t="inlineStr">
+      <c r="I88" s="7" t="inlineStr">
         <is>
           <t>潜在价值</t>
         </is>
       </c>
-      <c r="J85" s="5" t="inlineStr">
+      <c r="J88" s="5" t="inlineStr">
         <is>
           <t>市中心年年办的圣诞市集；2026 年日期只在官网看到，页面没更新干净</t>
         </is>
       </c>
-      <c r="K85" s="5" t="inlineStr">
+      <c r="K88" s="5" t="inlineStr">
         <is>
           <t>https://leicesterchristmasmarket.co.uk/</t>
         </is>
       </c>
-      <c r="L85" s="5" t="inlineStr">
+      <c r="L88" s="5" t="inlineStr">
         <is>
           <t>免费逛；推之前确认开市日期</t>
         </is>
       </c>
-      <c r="M85" s="5" t="inlineStr">
+      <c r="M88" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N85" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O85" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="58" customHeight="1">
-      <c r="A86" s="2" t="inlineStr">
+      <c r="N88" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O88" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="58" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>Staffs Student Life | Stoke / Keele Campus Life</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>待制作：Staffs Student Life | Stoke.png</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: STOKE 👇
@@ -6550,144 +6748,144 @@
 🎃 Trentham Halloween Festival, Stoke-on-Trent — last day of fire shows, pumpkin trail &amp; silent disco, 1 Nov.</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>Stoke-on-Trent Comedy Festival（含 Adam Kay、Hannah Byczkowski）</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>King's Hall, Glebe Street, Stoke-on-Trent ST4 1HH</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="G86" s="5" t="inlineStr">
+      <c r="G89" s="5" t="inlineStr">
         <is>
           <t>13–15 Nov 2026（Adam Kay：14 Nov 20:00）</t>
         </is>
       </c>
-      <c r="H86" s="5" t="inlineStr">
+      <c r="H89" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(喜剧)</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr">
+      <c r="I89" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J86" s="5" t="inlineStr">
+      <c r="J89" s="5" t="inlineStr">
         <is>
           <t>市政场馆 King's Hall 主办的喜剧节；Adam Kay（This Is Going to Hurt）是知名巡演喜剧人</t>
         </is>
       </c>
-      <c r="K86" s="5" t="inlineStr">
+      <c r="K89" s="5" t="inlineStr">
         <is>
           <t>https://www.stoke.gov.uk/kingshallevents ; https://www.songkick.com/metro-areas/24537-uk-stoke-on-trent/november-2026</t>
         </is>
       </c>
-      <c r="L86" s="5" t="inlineStr">
+      <c r="L89" s="5" t="inlineStr">
         <is>
           <t>周末喜剧节，有好几场可以选；Byczkowski 是《The Traitors》第一季冠军，话题度高</t>
         </is>
       </c>
-      <c r="M86" s="5" t="inlineStr">
+      <c r="M89" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N86" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O86" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="58" customHeight="1">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="3" t="n"/>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="N89" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O89" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="58" customHeight="1">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="4" t="n"/>
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Trentham Halloween Festival</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>Trentham Estate, Stone Road, Trentham, Stoke-on-Trent ST4 8JG</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="G87" s="5" t="inlineStr">
+      <c r="G90" s="5" t="inlineStr">
         <is>
           <t>31 Oct – 1 Nov 2026（窗口内只有 1 Nov）</t>
         </is>
       </c>
-      <c r="H87" s="5" t="inlineStr">
+      <c r="H90" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(万圣节/户外)</t>
         </is>
       </c>
-      <c r="I87" s="6" t="inlineStr">
+      <c r="I90" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J87" s="5" t="inlineStr">
+      <c r="J90" s="5" t="inlineStr">
         <is>
           <t>Trentham Estate 官方主办，Visit Staffordshire 收录；有火舞表演、南瓜灯小路、静音 disco</t>
         </is>
       </c>
-      <c r="K87" s="5" t="inlineStr">
+      <c r="K90" s="5" t="inlineStr">
         <is>
           <t>https://trentham.co.uk/events/trentham-halloween-festival/ ; https://www.visitstaffordshire.com/event/trentham-halloween-festival/234108101/</t>
         </is>
       </c>
-      <c r="L87" s="5" t="inlineStr">
+      <c r="L90" s="5" t="inlineStr">
         <is>
           <t>离 Keele、Staffs 都近；静音 disco 和火舞适合年轻人</t>
         </is>
       </c>
-      <c r="M87" s="5" t="inlineStr">
+      <c r="M90" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N87" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O87" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="71.5" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
+      <c r="N90" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O90" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="71.5" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>The University of Manchester / Manchester Metropolitan University</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>待制作：The University of Manchester.png</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: MANCHESTER 👇
@@ -6698,249 +6896,54 @@
 🎸 Blossoms, Co-op Live, Manchester — the local heroes' hometown arena show, 28 Nov.</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>Manchester Christmas Markets 2026</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>Albert Square / Cathedral Gardens / Exchange Square 等，Manchester city centre</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G88" s="5" t="inlineStr">
+      <c r="G91" s="5" t="inlineStr">
         <is>
           <t>6 Nov – 22 Dec 2026（窗口内为 6–30 Nov）</t>
         </is>
       </c>
-      <c r="H88" s="5" t="inlineStr">
+      <c r="H91" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市/美食)</t>
         </is>
       </c>
-      <c r="I88" s="8" t="inlineStr">
+      <c r="I91" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J88" s="5" t="inlineStr">
+      <c r="J91" s="5" t="inlineStr">
         <is>
           <t>年年举办的全英知名圣诞市集，The Manc 报道了 2026 年开市日期和新增点位</t>
         </is>
       </c>
-      <c r="K88" s="5" t="inlineStr">
+      <c r="K91" s="5" t="inlineStr">
         <is>
           <t>https://themanc.com/news/manchester-christmas-markets-2026-opening-date-announced-including-new-spots/ ; https://www.visitmanchester.com/whats-on/whats-on-this-christmas-in-manchester/</t>
         </is>
       </c>
-      <c r="L88" s="5" t="inlineStr">
+      <c r="L91" s="5" t="inlineStr">
         <is>
           <t>免费入场，市中心多个点位，逛吃一条龙</t>
         </is>
       </c>
-      <c r="M88" s="5" t="inlineStr">
+      <c r="M91" s="5" t="inlineStr">
         <is>
           <t>UK Food Lovers</t>
-        </is>
-      </c>
-      <c r="N88" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O88" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="58" customHeight="1">
-      <c r="A89" s="2" t="n"/>
-      <c r="B89" s="3" t="n"/>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>Manchester 市政免费烟花夜（Platt Fields / Heaton Park / Wythenshawe Park）</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>Platt Fields Park, Wilmslow Road, Fallowfield, Manchester M14 6LA（另有 Heaton Park、Wythenshawe Park 两个点）</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="inlineStr">
-        <is>
-          <t>7 Nov 2026（周六）17:00 低噪音场，20:00 主场烟花，之前有灯笼游行</t>
-        </is>
-      </c>
-      <c r="H89" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(烟花)</t>
-        </is>
-      </c>
-      <c r="I89" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J89" s="5" t="inlineStr">
-        <is>
-          <t>Manchester 市议会官方公布：市政烟花 2019 年后首次恢复；三个公园同时办</t>
-        </is>
-      </c>
-      <c r="K89" s="5" t="inlineStr">
-        <is>
-          <t>https://www.manchester.gov.uk/news-stories/2026/free-fireworks-night-events-to-make-spectacular-return-in-manchester</t>
-        </is>
-      </c>
-      <c r="L89" s="5" t="inlineStr">
-        <is>
-          <t>完全免费；Platt Fields 就在 Fallowfield 学生区，UoM 学生走路就到</t>
-        </is>
-      </c>
-      <c r="M89" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N89" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O89" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="58" customHeight="1">
-      <c r="A90" s="2" t="n"/>
-      <c r="B90" s="3" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>Northern Lights Manchester 灯光步道（主题：A Christmas Time Machine）</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Heaton Park, Middleton Road, Manchester M25 2SW</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>19 Nov – 31 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H90" s="5" t="inlineStr">
-        <is>
-          <t>本地生活类(灯光步道)</t>
-        </is>
-      </c>
-      <c r="I90" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J90" s="5" t="inlineStr">
-        <is>
-          <t>See Tickets 正规售票；今年新主题</t>
-        </is>
-      </c>
-      <c r="K90" s="5" t="inlineStr">
-        <is>
-          <t>https://northernlightsmanchester.seetickets.com/tour/northern-lights-manchester ; https://themanc.com/whats-on-manchester/northern-lights-trail-heaton-park-manchester/</t>
-        </is>
-      </c>
-      <c r="L90" s="5" t="inlineStr">
-        <is>
-          <t>peak 票 £17.50–25，off-peak £13.50–19.50，加 £1.75 手续费；选 off-peak 更划算</t>
-        </is>
-      </c>
-      <c r="M90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N90" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O90" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="58" customHeight="1">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="3" t="n"/>
-      <c r="C91" s="4" t="n"/>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>Phoebe Bridgers 演唱会（嘉宾 Isaac Wood、Anaïs）</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>Co-op Live, Etihad Campus, Manchester</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>venue_only</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
-        <is>
-          <t>26 Nov 2026（周四）</t>
-        </is>
-      </c>
-      <c r="H91" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/独立)</t>
-        </is>
-      </c>
-      <c r="I91" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J91" s="5" t="inlineStr">
-        <is>
-          <t>Co-op Live 场馆日程和 Stereoboard 都列出；只看到列表信息，还没看到单场票务页</t>
-        </is>
-      </c>
-      <c r="K91" s="5" t="inlineStr">
-        <is>
-          <t>https://www.cooplive.com/ ; https://www.stereoboard.com/venues/manchester/co-op-live</t>
-        </is>
-      </c>
-      <c r="L91" s="5" t="inlineStr">
-        <is>
-          <t>独立乐迷的大场；推之前确认一下票务页</t>
-        </is>
-      </c>
-      <c r="M91" s="5" t="inlineStr">
-        <is>
-          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="N91" s="5" t="inlineStr">
@@ -6960,77 +6963,272 @@
       <c r="C92" s="4" t="n"/>
       <c r="D92" s="2" t="inlineStr">
         <is>
+          <t>Manchester 市政免费烟花夜（Platt Fields / Heaton Park / Wythenshawe Park）</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Platt Fields Park, Wilmslow Road, Fallowfield, Manchester M14 6LA（另有 Heaton Park、Wythenshawe Park 两个点）</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）17:00 低噪音场，20:00 主场烟花，之前有灯笼游行</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>Manchester 市议会官方公布：市政烟花 2019 年后首次恢复；三个公园同时办</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="inlineStr">
+        <is>
+          <t>https://www.manchester.gov.uk/news-stories/2026/free-fireworks-night-events-to-make-spectacular-return-in-manchester</t>
+        </is>
+      </c>
+      <c r="L92" s="5" t="inlineStr">
+        <is>
+          <t>完全免费；Platt Fields 就在 Fallowfield 学生区，UoM 学生走路就到</t>
+        </is>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N92" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O92" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="58" customHeight="1">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="4" t="n"/>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Northern Lights Manchester 灯光步道（主题：A Christmas Time Machine）</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Heaton Park, Middleton Road, Manchester M25 2SW</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>19 Nov – 31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>本地生活类(灯光步道)</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>See Tickets 正规售票；今年新主题</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>https://northernlightsmanchester.seetickets.com/tour/northern-lights-manchester ; https://themanc.com/whats-on-manchester/northern-lights-trail-heaton-park-manchester/</t>
+        </is>
+      </c>
+      <c r="L93" s="5" t="inlineStr">
+        <is>
+          <t>peak 票 £17.50–25，off-peak £13.50–19.50，加 £1.75 手续费；选 off-peak 更划算</t>
+        </is>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N93" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O93" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="58" customHeight="1">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="4" t="n"/>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Phoebe Bridgers 演唱会（嘉宾 Isaac Wood、Anaïs）</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Co-op Live, Etihad Campus, Manchester</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>26 Nov 2026（周四）</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立)</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>Co-op Live 场馆日程和 Stereoboard 都列出；只看到列表信息，还没看到单场票务页</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cooplive.com/ ; https://www.stereoboard.com/venues/manchester/co-op-live</t>
+        </is>
+      </c>
+      <c r="L94" s="5" t="inlineStr">
+        <is>
+          <t>独立乐迷的大场；推之前确认一下票务页</t>
+        </is>
+      </c>
+      <c r="M94" s="5" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="N94" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O94" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="58" customHeight="1">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
           <t>Blossoms 演唱会（嘉宾 The Royston Club）</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>Co-op Live, Etihad Campus, Manchester</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="F95" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G92" s="5" t="inlineStr">
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>28 Nov 2026（周六）</t>
         </is>
       </c>
-      <c r="H92" s="5" t="inlineStr">
+      <c r="H95" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(Live Music/英伦独立)</t>
         </is>
       </c>
-      <c r="I92" s="6" t="inlineStr">
+      <c r="I95" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J92" s="5" t="inlineStr">
+      <c r="J95" s="5" t="inlineStr">
         <is>
           <t>Co-op Live 场馆日程列出；Blossoms 是大曼彻斯特本地乐队，主场演出</t>
         </is>
       </c>
-      <c r="K92" s="5" t="inlineStr">
+      <c r="K95" s="5" t="inlineStr">
         <is>
           <t>https://www.cooplive.com/ ; https://www.jambase.com/venue/co-op-live-arena</t>
         </is>
       </c>
-      <c r="L92" s="5" t="inlineStr">
+      <c r="L95" s="5" t="inlineStr">
         <is>
           <t>本地乐队的主场大秀，周六晚上</t>
         </is>
       </c>
-      <c r="M92" s="5" t="inlineStr">
+      <c r="M95" s="5" t="inlineStr">
         <is>
           <t>Live Music Crew</t>
         </is>
       </c>
-      <c r="N92" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O92" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="58" customHeight="1">
-      <c r="A93" s="2" t="inlineStr">
+      <c r="N95" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O95" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="58" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>University of Lancaster</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>待制作：University of Lancaster.png</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: LANCASTER &amp; THE LAKES 👇
@@ -7038,144 +7236,144 @@
 💡 Light Up Lancaster, Lancaster — a free light-art trail across the city, 5–7 Nov.</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>Kendal Mountain Festival 2026（户外电影 + 讲座 + 文学）</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>Kendal, Cumbria（多个场地，节目单见 kendalmountainfestival.com）</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>city_only</t>
         </is>
       </c>
-      <c r="G93" s="5" t="inlineStr">
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>19–22 Nov 2026（周四到周日）</t>
         </is>
       </c>
-      <c r="H93" s="5" t="inlineStr">
+      <c r="H96" s="5" t="inlineStr">
         <is>
           <t>运动户外 + 电影/媒体</t>
         </is>
       </c>
-      <c r="I93" s="8" t="inlineStr">
+      <c r="I96" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J93" s="5" t="inlineStr">
+      <c r="J96" s="5" t="inlineStr">
         <is>
           <t>英国最大的户外山地节：200 多场活动、300 多位讲者、150 多部电影、10 多场派对（主办方数据）；年年举办</t>
         </is>
       </c>
-      <c r="K93" s="5" t="inlineStr">
+      <c r="K96" s="5" t="inlineStr">
         <is>
           <t>https://www.kendalmountainfestival.com/ ; https://kendalbid.co.uk/event/kendal-mountain-festival-2026/</t>
         </is>
       </c>
-      <c r="L93" s="5" t="inlineStr">
+      <c r="L96" s="5" t="inlineStr">
         <is>
           <t>户外迷必去；离 Lancaster 约 35 公里，火车可达；也有线上片单</t>
         </is>
       </c>
-      <c r="M93" s="5" t="inlineStr">
+      <c r="M96" s="5" t="inlineStr">
         <is>
           <t>Day Trip Buddies；Reel Talk Club；Outdoor Adventure Club</t>
         </is>
       </c>
-      <c r="N93" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O93" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="71.5" customHeight="1">
-      <c r="A94" s="2" t="n"/>
-      <c r="B94" s="3" t="n"/>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="N96" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O96" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="71.5" customHeight="1">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="4" t="n"/>
+      <c r="D97" s="2" t="inlineStr">
         <is>
           <t>Light Up Lancaster 2026（主题：No Boundaries）</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
+      <c r="E97" s="2" t="inlineStr">
         <is>
           <t>Lancaster city centre：Market Square、Dalton Square、The Storey Gardens、Lancaster Castle、Quay Meadow 等（完整地图见 lightuplancaster.co.uk）</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>5–7 Nov 2026（周四到周六）17:00–22:00</t>
         </is>
       </c>
-      <c r="H94" s="5" t="inlineStr">
+      <c r="H97" s="5" t="inlineStr">
         <is>
           <t>本地生活类(灯光艺术节)</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr">
+      <c r="I97" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J94" s="5" t="inlineStr">
+      <c r="J97" s="5" t="inlineStr">
         <is>
           <t>Light Up the North 联盟成员，年年举办；Lancaster BID、Visit Lancashire、Lancaster Guardian、Beyond Radio 都有报道</t>
         </is>
       </c>
-      <c r="K94" s="5" t="inlineStr">
+      <c r="K97" s="5" t="inlineStr">
         <is>
           <t>https://www.lightuplancaster.co.uk/ ; https://www.beyond.radio/news/local-news/light-up-lancaster-promises-to-illuminate-city-with-no-boundaries/ ; https://www.facebook.com/lightuplancaster/</t>
         </is>
       </c>
-      <c r="L94" s="5" t="inlineStr">
+      <c r="L97" s="5" t="inlineStr">
         <is>
           <t>免费的灯光艺术路线，连着三晚，下课后去逛正合适</t>
         </is>
       </c>
-      <c r="M94" s="5" t="inlineStr">
+      <c r="M97" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N94" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O94" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="58" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
+      <c r="N97" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O97" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="58" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>University of Lancashire</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>待制作：University of Lancashire.png</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: PRESTON 👇
@@ -7183,223 +7381,223 @@
 🦢 Swan feeds at WWT Martin Mere, Burscough, Lancashire — up to 2,000 whooper swans (times TBC), daily from Nov.</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>Preston 圣诞亮灯（East 17 压轴）</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>Flag Market, Preston city centre</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G95" s="5" t="inlineStr">
+      <c r="G98" s="5" t="inlineStr">
         <is>
           <t>21 Nov 2026（周六）17:00 起</t>
         </is>
       </c>
-      <c r="H95" s="5" t="inlineStr">
+      <c r="H98" s="5" t="inlineStr">
         <is>
           <t>本地生活类(节庆/音乐)</t>
         </is>
       </c>
-      <c r="I95" s="6" t="inlineStr">
+      <c r="I98" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J95" s="5" t="inlineStr">
+      <c r="J98" s="5" t="inlineStr">
         <is>
           <t>Preston BID 和 Smooth Radio 主办，LEP 报道、Visit Preston 列出；另一个页面写 22 Nov（是 2025 年的日期）</t>
         </is>
       </c>
-      <c r="K95" s="5" t="inlineStr">
+      <c r="K98" s="5" t="inlineStr">
         <is>
           <t>https://www.lep.co.uk/news/east-17-to-headline-prestons-chirstmas-lights-switch-on-9276860 ; https://www.visitpreston.com/article/8354/Christmas-Lights-Switch-On-2026</t>
         </is>
       </c>
-      <c r="L95" s="5" t="inlineStr">
+      <c r="L98" s="5" t="inlineStr">
         <is>
           <t>免费；University of Lancashire 主校区就在市中心</t>
         </is>
       </c>
-      <c r="M95" s="5" t="inlineStr">
+      <c r="M98" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N95" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O95" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="58" customHeight="1">
-      <c r="A96" s="2" t="n"/>
-      <c r="B96" s="3" t="n"/>
-      <c r="C96" s="4" t="n"/>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="N98" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O98" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="58" customHeight="1">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="4" t="n"/>
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>WWT Martin Mere 冬季天鹅喂食秀</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>WWT Martin Mere Wetland Centre, Fish Lane, Burscough, Lancashire</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G96" s="5" t="inlineStr">
+      <c r="G99" s="5" t="inlineStr">
         <is>
           <t>⚠️11 月起每天（往年 15:00、15:30 两场，2026 年时间表还没公布）</t>
         </is>
       </c>
-      <c r="H96" s="5" t="inlineStr">
+      <c r="H99" s="5" t="inlineStr">
         <is>
           <t>兴趣类(观鸟)</t>
         </is>
       </c>
-      <c r="I96" s="7" t="inlineStr">
+      <c r="I99" s="7" t="inlineStr">
         <is>
           <t>潜在价值</t>
         </is>
       </c>
-      <c r="J96" s="5" t="inlineStr">
+      <c r="J99" s="5" t="inlineStr">
         <is>
           <t>WWT 官网往年介绍：最多约 2,000 只大天鹅来吃食；2026 年时间表没找到</t>
         </is>
       </c>
-      <c r="K96" s="5" t="inlineStr">
+      <c r="K99" s="5" t="inlineStr">
         <is>
           <t>https://www.wwt.org.uk/wetland-centres/martin-mere/news/have-a-wild-winter-at-martin-mere-wetland-centre</t>
         </is>
       </c>
-      <c r="L96" s="5" t="inlineStr">
+      <c r="L99" s="5" t="inlineStr">
         <is>
           <t>离 Preston 约 25 公里；去之前查一下当天喂食时间</t>
         </is>
       </c>
-      <c r="M96" s="5" t="inlineStr">
+      <c r="M99" s="5" t="inlineStr">
         <is>
           <t>Birdwatch Brigade</t>
         </is>
       </c>
-      <c r="N96" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O96" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="60" customHeight="1">
-      <c r="A97" s="2" t="inlineStr">
+      <c r="N99" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O99" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="60" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>University of Chester</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B100" s="3" t="inlineStr">
         <is>
           <t>待制作：University of Chester.png</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: CHESTER 👇
 🎄 Chester Christmas Market, Town Hall Square — 80 stalls inside the old city walls, from 18 Nov.</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>Chester Christmas Market</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>Town Hall Square, Northgate Street, Chester CH1 2HJ</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="G97" s="5" t="inlineStr">
+      <c r="G100" s="5" t="inlineStr">
         <is>
           <t>18 Nov – 22 Dec 2026（周日到周三 10:30–18:30，周四到周六到 20:00）</t>
         </is>
       </c>
-      <c r="H97" s="5" t="inlineStr">
+      <c r="H100" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市)</t>
         </is>
       </c>
-      <c r="I97" s="6" t="inlineStr">
+      <c r="I100" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J97" s="5" t="inlineStr">
+      <c r="J100" s="5" t="inlineStr">
         <is>
           <t>官网和 Visit Cheshire、Visit Chester 日期一致；约 80 个摊位</t>
         </is>
       </c>
-      <c r="K97" s="5" t="inlineStr">
+      <c r="K100" s="5" t="inlineStr">
         <is>
           <t>https://chester-christmasmarket.com/ ; https://visitcheshire.com/events/chester-christmas-market</t>
         </is>
       </c>
-      <c r="L97" s="5" t="inlineStr">
+      <c r="L100" s="5" t="inlineStr">
         <is>
           <t>免费；古城墙加圣诞市集，切斯特这个月最好的选择</t>
         </is>
       </c>
-      <c r="M97" s="5" t="inlineStr">
+      <c r="M100" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N97" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O97" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="71.5" customHeight="1">
-      <c r="A98" s="2" t="inlineStr">
+      <c r="N100" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O100" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="71.5" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>Leeds Uni Student Hub / Leeds University group 2 / Leeds University group 3 / Leeds University group 4 / Leeds University group 5 / Leeds University group 6 / Leeds University group 7</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B101" s="3" t="inlineStr">
         <is>
           <t>待制作：Leeds Uni Student Hub.png</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: LEEDS 👇
@@ -7411,249 +7609,54 @@
 🎄 Leeds Christmas Market &amp; Ice Cube, City Square &amp; Millennium Square — festive stalls plus a skating rink, from 19 Nov.</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t>Leeds International Film Festival（第 40 届）</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E101" s="2" t="inlineStr">
         <is>
           <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G98" s="5" t="inlineStr">
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>29 Oct – 15 Nov 2026（窗口内为 1–15 Nov）</t>
         </is>
       </c>
-      <c r="H98" s="5" t="inlineStr">
+      <c r="H101" s="5" t="inlineStr">
         <is>
           <t>电影/媒体</t>
         </is>
       </c>
-      <c r="I98" s="8" t="inlineStr">
+      <c r="I101" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J98" s="5" t="inlineStr">
+      <c r="J101" s="5" t="inlineStr">
         <is>
           <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
         </is>
       </c>
-      <c r="K98" s="5" t="inlineStr">
+      <c r="K101" s="5" t="inlineStr">
         <is>
           <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
         </is>
       </c>
-      <c r="L98" s="5" t="inlineStr">
+      <c r="L101" s="5" t="inlineStr">
         <is>
           <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
         </is>
       </c>
-      <c r="M98" s="5" t="inlineStr">
+      <c r="M101" s="5" t="inlineStr">
         <is>
           <t>Reel Talk Club</t>
-        </is>
-      </c>
-      <c r="N98" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O98" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="58" customHeight="1">
-      <c r="A99" s="2" t="n"/>
-      <c r="B99" s="3" t="n"/>
-      <c r="C99" s="4" t="n"/>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>Leeds Abbey Dash 10K</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>起终点 Wellington Street, Leeds LS1 4DL（路线往返 Kirkstall Abbey）</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>29 Nov 2026（周日）9:30 起跑</t>
-        </is>
-      </c>
-      <c r="H99" s="5" t="inlineStr">
-        <is>
-          <t>运动户外(跑步)</t>
-        </is>
-      </c>
-      <c r="I99" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J99" s="5" t="inlineStr">
-        <is>
-          <t>利兹老牌 10K，办了近 40 年；今年是英格兰田径 10K 锦标赛指定赛事；Run For All 主办</t>
-        </is>
-      </c>
-      <c r="K99" s="5" t="inlineStr">
-        <is>
-          <t>https://www.runforall.com/events/10k/abbey-dash/ ; https://www.runforall.com/community/news/leeds-abbey-dash-2026-opens-for-entries-as-england-athletics-championship-returns/</t>
-        </is>
-      </c>
-      <c r="L99" s="5" t="inlineStr">
-        <is>
-          <t>报名费约 £29–41（看渠道）；路线平坦，适合第一次跑 10K</t>
-        </is>
-      </c>
-      <c r="M99" s="5" t="inlineStr">
-        <is>
-          <t>Fitness Check-ins</t>
-        </is>
-      </c>
-      <c r="N99" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O99" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="58" customHeight="1">
-      <c r="A100" s="2" t="n"/>
-      <c r="B100" s="3" t="n"/>
-      <c r="C100" s="4" t="n"/>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>Jungle 演唱会</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>first direct bank arena, Arena Way, Leeds LS2 8BY</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>21 Nov 2026（周六）18:30/19:00</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/电子灵魂)</t>
-        </is>
-      </c>
-      <c r="I100" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J100" s="5" t="inlineStr">
-        <is>
-          <t>See Tickets、AXS、Ticketmaster 正规售票；二手票溢价到 £140 以上，说明需求旺</t>
-        </is>
-      </c>
-      <c r="K100" s="5" t="inlineStr">
-        <is>
-          <t>https://www.seetickets.com/event/jungle/first-direct-bank-arena/3618943 ; https://www.axs.com/uk/events/1383202/jungle-tickets</t>
-        </is>
-      </c>
-      <c r="L100" s="5" t="inlineStr">
-        <is>
-          <t>票面 £40 起，别买二手高价票；体育场离 Leeds 大学走路 10 分钟</t>
-        </is>
-      </c>
-      <c r="M100" s="5" t="inlineStr">
-        <is>
-          <t>Live Music Crew</t>
-        </is>
-      </c>
-      <c r="N100" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O100" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="58" customHeight="1">
-      <c r="A101" s="2" t="n"/>
-      <c r="B101" s="3" t="n"/>
-      <c r="C101" s="4" t="n"/>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr">
-        <is>
-          <t>13 Nov 2026（周五）19:00</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
-        </is>
-      </c>
-      <c r="I101" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J101" s="5" t="inlineStr">
-        <is>
-          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
-        </is>
-      </c>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
-        </is>
-      </c>
-      <c r="L101" s="5" t="inlineStr">
-        <is>
-          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
-        </is>
-      </c>
-      <c r="M101" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
       <c r="N101" s="5" t="inlineStr">
@@ -7673,12 +7676,12 @@
       <c r="C102" s="4" t="n"/>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Northern Lights Leeds 灯光步道</t>
+          <t>Leeds Abbey Dash 10K</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Temple Newsam, Temple Newsam Road, Leeds LS15 0AE</t>
+          <t>起终点 Wellington Street, Leeds LS1 4DL（路线往返 Kirkstall Abbey）</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -7688,37 +7691,37 @@
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>20 Nov – 31 Dec 2026，16:15 起入场</t>
+          <t>29 Nov 2026（周日）9:30 起跑</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>本地生活类(灯光步道)</t>
-        </is>
-      </c>
-      <c r="I102" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
+          <t>运动户外(跑步)</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>See Tickets 正规售票，2026 年有官方日期；主办方写明日期可能调整</t>
+          <t>利兹老牌 10K，办了近 40 年；今年是英格兰田径 10K 锦标赛指定赛事；Run For All 主办</t>
         </is>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>https://northernlightsleeds.seetickets.com/ ; https://www.yorkshireeveningpost.co.uk/whats-on/northern-lights-leeds-temple-newsam-lost-light-of-christmas-preview-map-8985967</t>
+          <t>https://www.runforall.com/events/10k/abbey-dash/ ; https://www.runforall.com/community/news/leeds-abbey-dash-2026-opens-for-entries-as-england-athletics-championship-returns/</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
         <is>
-          <t>分时段入场；Temple Newsam 在城东，要坐公交</t>
+          <t>报名费约 £29–41（看渠道）；路线平坦，适合第一次跑 10K</t>
         </is>
       </c>
       <c r="M102" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fitness Check-ins</t>
         </is>
       </c>
       <c r="N102" s="5" t="inlineStr">
@@ -7738,127 +7741,112 @@
       <c r="C103" s="4" t="n"/>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Leeds Christmas Market + Ice Cube 溜冰场</t>
+          <t>Jungle 演唱会</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>City Square（市集）/ Millennium Square（Ice Cube）, Leeds city centre</t>
+          <t>first direct bank arena, Arena Way, Leeds LS2 8BY</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>19 Nov – 23 Dec 2026（Ice Cube 开始日期有 19 Nov 和 22 Nov 两种说法）</t>
+          <t>21 Nov 2026（周六）18:30/19:00</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>本地生活类(集市/滑冰)</t>
-        </is>
-      </c>
-      <c r="I103" s="6" t="inlineStr">
+          <t>年轻人娱乐(Live Music/电子灵魂)</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J103" s="5" t="inlineStr">
+        <is>
+          <t>See Tickets、AXS、Ticketmaster 正规售票；二手票溢价到 £140 以上，说明需求旺</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>https://www.seetickets.com/event/jungle/first-direct-bank-arena/3618943 ; https://www.axs.com/uk/events/1383202/jungle-tickets</t>
+        </is>
+      </c>
+      <c r="L103" s="5" t="inlineStr">
+        <is>
+          <t>票面 £40 起，别买二手高价票；体育场离 Leeds 大学走路 10 分钟</t>
+        </is>
+      </c>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="N103" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O103" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="58" customHeight="1">
+      <c r="A104" s="2" t="n"/>
+      <c r="B104" s="3" t="n"/>
+      <c r="C104" s="4" t="n"/>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>13 Nov 2026（周五）19:00</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
+        </is>
+      </c>
+      <c r="I104" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J103" s="5" t="inlineStr">
-        <is>
-          <t>LNER、Visit Chester 等多个来源列出 2026 年日期；部分细节主办方还在定</t>
-        </is>
-      </c>
-      <c r="K103" s="5" t="inlineStr">
-        <is>
-          <t>https://www.lner.co.uk/destinations/travel-inspiration/christmas-markets-and-festive-events/trains-to-leeds-christmas-market/ ; https://www.leedschristmas.co.uk/</t>
-        </is>
-      </c>
-      <c r="L103" s="5" t="inlineStr">
-        <is>
-          <t>免费逛市集；溜冰场在 Millennium Square，离 Leeds 大学很近</t>
-        </is>
-      </c>
-      <c r="M103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O103" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="58" customHeight="1">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Sheffield Hallam University / University of Sheffield</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>待制作：Sheffield Hallam University.png</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="inlineStr">
-        <is>
-          <t>🔍 Event Radar (UK) — what's worth doing this month.
-This month: SHEFFIELD 👇
-🎆 ArcNight, Don Valley Bowl, Sheffield — Sheffield's big Bonfire Night show, 5 Nov.
-🎄 Sheffield Christmas Market, Fargate &amp; The Moor — festive cabins in the city centre, from 12 Nov.</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>ArcNight 2026：谢菲尔德篝火夜烟花</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>Don Valley Bowl, Coleridge Road, Sheffield S9 2DF</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>5 Nov 2026（周四）16:00–21:00</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(烟花)</t>
-        </is>
-      </c>
-      <c r="I104" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
       <c r="J104" s="5" t="inlineStr">
         <is>
-          <t>新办的活动，由 Illuminate the Gardens 团队主办；Exposed Magazine、Yorkshire Live 报道；票价还没公布</t>
+          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
         </is>
       </c>
       <c r="K104" s="5" t="inlineStr">
         <is>
-          <t>https://arcnight.com/ ; https://www.exposedmagazine.co.uk/whats-new/brand-new-bonfire-night-spectacular-to-bring-sheffield-steel-to-the-sky-at-don-valley/</t>
+          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
         </is>
       </c>
       <c r="L104" s="5" t="inlineStr">
         <is>
-          <t>谢菲尔德唯一的大型烟花，篝火夜正日子；有电车可以到</t>
+          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
         </is>
       </c>
       <c r="M104" s="5" t="inlineStr">
@@ -7883,77 +7871,287 @@
       <c r="C105" s="4" t="n"/>
       <c r="D105" s="2" t="inlineStr">
         <is>
+          <t>Northern Lights Leeds 灯光步道</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Temple Newsam, Temple Newsam Road, Leeds LS15 0AE</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>20 Nov – 31 Dec 2026，16:15 起入场</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>本地生活类(灯光步道)</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J105" s="5" t="inlineStr">
+        <is>
+          <t>See Tickets 正规售票，2026 年有官方日期；主办方写明日期可能调整</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>https://northernlightsleeds.seetickets.com/ ; https://www.yorkshireeveningpost.co.uk/whats-on/northern-lights-leeds-temple-newsam-lost-light-of-christmas-preview-map-8985967</t>
+        </is>
+      </c>
+      <c r="L105" s="5" t="inlineStr">
+        <is>
+          <t>分时段入场；Temple Newsam 在城东，要坐公交</t>
+        </is>
+      </c>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N105" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O105" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="58" customHeight="1">
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="3" t="n"/>
+      <c r="C106" s="4" t="n"/>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Leeds Christmas Market + Ice Cube 溜冰场</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>City Square（市集）/ Millennium Square（Ice Cube）, Leeds city centre</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>19 Nov – 23 Dec 2026（Ice Cube 开始日期有 19 Nov 和 22 Nov 两种说法）</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>本地生活类(集市/滑冰)</t>
+        </is>
+      </c>
+      <c r="I106" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>LNER、Visit Chester 等多个来源列出 2026 年日期；部分细节主办方还在定</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>https://www.lner.co.uk/destinations/travel-inspiration/christmas-markets-and-festive-events/trains-to-leeds-christmas-market/ ; https://www.leedschristmas.co.uk/</t>
+        </is>
+      </c>
+      <c r="L106" s="5" t="inlineStr">
+        <is>
+          <t>免费逛市集；溜冰场在 Millennium Square，离 Leeds 大学很近</t>
+        </is>
+      </c>
+      <c r="M106" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N106" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O106" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="58" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Sheffield Hallam University / University of Sheffield</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>待制作：Sheffield Hallam University.png</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>🔍 Event Radar (UK) — what's worth doing this month.
+This month: SHEFFIELD 👇
+🎆 ArcNight, Don Valley Bowl, Sheffield — Sheffield's big Bonfire Night show, 5 Nov.
+🎄 Sheffield Christmas Market, Fargate &amp; The Moor — festive cabins in the city centre, from 12 Nov.</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>ArcNight 2026：谢菲尔德篝火夜烟花</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Don Valley Bowl, Coleridge Road, Sheffield S9 2DF</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>5 Nov 2026（周四）16:00–21:00</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
+        <is>
+          <t>新办的活动，由 Illuminate the Gardens 团队主办；Exposed Magazine、Yorkshire Live 报道；票价还没公布</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="inlineStr">
+        <is>
+          <t>https://arcnight.com/ ; https://www.exposedmagazine.co.uk/whats-new/brand-new-bonfire-night-spectacular-to-bring-sheffield-steel-to-the-sky-at-don-valley/</t>
+        </is>
+      </c>
+      <c r="L107" s="5" t="inlineStr">
+        <is>
+          <t>谢菲尔德唯一的大型烟花，篝火夜正日子；有电车可以到</t>
+        </is>
+      </c>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N107" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O107" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="58" customHeight="1">
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="4" t="n"/>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
           <t>Sheffield Christmas Market</t>
         </is>
       </c>
-      <c r="E105" s="2" t="inlineStr">
+      <c r="E108" s="2" t="inlineStr">
         <is>
           <t>Fargate / Pinstone Street / The Moor, Sheffield city centre</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr">
+      <c r="F108" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G108" s="5" t="inlineStr">
         <is>
           <t>12 Nov – 26 Dec 2026</t>
         </is>
       </c>
-      <c r="H105" s="5" t="inlineStr">
+      <c r="H108" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市)</t>
         </is>
       </c>
-      <c r="I105" s="6" t="inlineStr">
+      <c r="I108" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J105" s="5" t="inlineStr">
+      <c r="J108" s="5" t="inlineStr">
         <is>
           <t>Welcome to Sheffield 官方列出 2026 年日期；市政亮灯仪式 2023 年起停办，今年还没确认</t>
         </is>
       </c>
-      <c r="K105" s="5" t="inlineStr">
+      <c r="K108" s="5" t="inlineStr">
         <is>
           <t>https://www.welcometosheffield.co.uk/content/events/sheffield-christmas-market-2026</t>
         </is>
       </c>
-      <c r="L105" s="5" t="inlineStr">
+      <c r="L108" s="5" t="inlineStr">
         <is>
           <t>免费逛；Hallam 城市校区就在旁边</t>
         </is>
       </c>
-      <c r="M105" s="5" t="inlineStr">
+      <c r="M108" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N105" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O105" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="58" customHeight="1">
-      <c r="A106" s="2" t="inlineStr">
+      <c r="N108" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O108" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="58" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>Huddersfield Uni Student Hub</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>待制作：Huddersfield Uni Student Hub.png</t>
         </is>
       </c>
-      <c r="C106" s="4" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: HUDDERSFIELD 👇
@@ -7962,264 +8160,54 @@
 🎆 Mirfield Bonfire &amp; Firework Extravaganza, Mirfield — bonfire, music stage and funfair, 7 Nov.</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
+      <c r="D109" s="2" t="inlineStr">
         <is>
           <t>hcmf// 哈德斯菲尔德当代音乐节（第 49 届）</t>
         </is>
       </c>
-      <c r="E106" s="2" t="inlineStr">
+      <c r="E109" s="2" t="inlineStr">
         <is>
           <t>Huddersfield 多个场地（官网节目单分场馆列出）</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr">
+      <c r="F109" s="2" t="inlineStr">
         <is>
           <t>city_only</t>
         </is>
       </c>
-      <c r="G106" s="5" t="inlineStr">
+      <c r="G109" s="5" t="inlineStr">
         <is>
           <t>20–29 Nov 2026</t>
         </is>
       </c>
-      <c r="H106" s="5" t="inlineStr">
+      <c r="H109" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(Live Music/实验音乐)</t>
         </is>
       </c>
-      <c r="I106" s="8" t="inlineStr">
+      <c r="I109" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J106" s="5" t="inlineStr">
+      <c r="J109" s="5" t="inlineStr">
         <is>
           <t>英国最重要的当代和实验音乐节，第 49 届，70 多场首演；官网已开票</t>
         </is>
       </c>
-      <c r="K106" s="5" t="inlineStr">
+      <c r="K109" s="5" t="inlineStr">
         <is>
           <t>https://hcmf.co.uk/hcmf-2026-now-on-sale/ ; https://hcmf.co.uk/2026-programme/</t>
         </is>
       </c>
-      <c r="L106" s="5" t="inlineStr">
+      <c r="L109" s="5" t="inlineStr">
         <is>
           <t>音乐专业学生必去；有讲座、装置和工作坊，部分场次免费</t>
         </is>
       </c>
-      <c r="M106" s="5" t="inlineStr">
+      <c r="M109" s="5" t="inlineStr">
         <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="N106" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O106" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="58" customHeight="1">
-      <c r="A107" s="2" t="n"/>
-      <c r="B107" s="3" t="n"/>
-      <c r="C107" s="4" t="n"/>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>Huddersfield &amp; District Round Table 慈善篝火烟花夜</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>DRAM Sport &amp; Community Centre, Ridgeway, Dalton, Huddersfield HD5 9QJ</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr">
-        <is>
-          <t>7 Nov 2026（周六）17:00 开门</t>
-        </is>
-      </c>
-      <c r="H107" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(烟花)</t>
-        </is>
-      </c>
-      <c r="I107" s="7" t="inlineStr">
-        <is>
-          <t>潜在价值</t>
-        </is>
-      </c>
-      <c r="J107" s="5" t="inlineStr">
-        <is>
-          <t>Yorkshire Live 列入约克郡篝火夜推荐；本地慈善机构年年办；没有售票数据</t>
-        </is>
-      </c>
-      <c r="K107" s="5" t="inlineStr">
-        <is>
-          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
-        </is>
-      </c>
-      <c r="L107" s="5" t="inlineStr">
-        <is>
-          <t>成人 £5，很便宜，离市中心近</t>
-        </is>
-      </c>
-      <c r="M107" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N107" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O107" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="58" customHeight="1">
-      <c r="A108" s="2" t="n"/>
-      <c r="B108" s="3" t="n"/>
-      <c r="C108" s="4" t="n"/>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>Mirfield Bonfire &amp; Firework Extravaganza</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>Mirfield Showground, Huddersfield Road, Mirfield WF14 9NE</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G108" s="5" t="inlineStr">
-        <is>
-          <t>7 Nov 2026（周六）16:00 开门，约 19:30 放烟花</t>
-        </is>
-      </c>
-      <c r="H108" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
-        </is>
-      </c>
-      <c r="I108" s="7" t="inlineStr">
-        <is>
-          <t>潜在价值</t>
-        </is>
-      </c>
-      <c r="J108" s="5" t="inlineStr">
-        <is>
-          <t>Yorkshire Live 列入约克郡最大篝火夜之一；有音乐舞台和游乐场；没有售票数据</t>
-        </is>
-      </c>
-      <c r="K108" s="5" t="inlineStr">
-        <is>
-          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
-        </is>
-      </c>
-      <c r="L108" s="5" t="inlineStr">
-        <is>
-          <t>离 Huddersfield 约 10 公里，比市内的活动规模大</t>
-        </is>
-      </c>
-      <c r="M108" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N108" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O108" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="58" customHeight="1">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>university of york student hub</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>待制作：university of york student hub.png</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>🔍 Event Radar (UK) — what's worth doing this month.
-This month: YORK 👇
-🎄 York Christmas Market, Parliament Street, York — one of the UK's best festive markets (closed Tuesdays), from 12 Nov.
-🌿 RHS Glow at Harlow Carr, Harrogate — a garden lit up for its 10th year, from 26 Nov.</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>York Christmas Market（St Nicholas Fair）</t>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>Parliament Street &amp; St Sampson's Square, York YO1</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>venue_only</t>
-        </is>
-      </c>
-      <c r="G109" s="5" t="inlineStr">
-        <is>
-          <t>12 Nov – 21 Dec 2026，10:30–19:00（周二不开，今年试行）</t>
-        </is>
-      </c>
-      <c r="H109" s="5" t="inlineStr">
-        <is>
-          <t>本地生活类(集市) + 一日游</t>
-        </is>
-      </c>
-      <c r="I109" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J109" s="5" t="inlineStr">
-        <is>
-          <t>Make It York 官方公布 2026 年日期和营业时间；英国最有名的圣诞市集之一</t>
-        </is>
-      </c>
-      <c r="K109" s="5" t="inlineStr">
-        <is>
-          <t>https://www.makeityork.com/news/2026/08/york-christmas-market-2026-dates-announced/ ; https://visityork.org/christmas/york-christmas-market</t>
-        </is>
-      </c>
-      <c r="L109" s="5" t="inlineStr">
-        <is>
-          <t>免费；⚠️周二不开；古城加圣诞市集，很适合一日游</t>
-        </is>
-      </c>
-      <c r="M109" s="5" t="inlineStr">
-        <is>
-          <t>Day Trip Buddies</t>
         </is>
       </c>
       <c r="N109" s="5" t="inlineStr">
@@ -8239,156 +8227,366 @@
       <c r="C110" s="4" t="n"/>
       <c r="D110" s="2" t="inlineStr">
         <is>
+          <t>Huddersfield &amp; District Round Table 慈善篝火烟花夜</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>DRAM Sport &amp; Community Centre, Ridgeway, Dalton, Huddersfield HD5 9QJ</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）17:00 开门</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="I110" s="7" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="J110" s="5" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡篝火夜推荐；本地慈善机构年年办；没有售票数据</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="L110" s="5" t="inlineStr">
+        <is>
+          <t>成人 £5，很便宜，离市中心近</t>
+        </is>
+      </c>
+      <c r="M110" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O110" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="58" customHeight="1">
+      <c r="A111" s="2" t="n"/>
+      <c r="B111" s="3" t="n"/>
+      <c r="C111" s="4" t="n"/>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Bonfire &amp; Firework Extravaganza</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Showground, Huddersfield Road, Mirfield WF14 9NE</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）16:00 开门，约 19:30 放烟花</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/音乐)</t>
+        </is>
+      </c>
+      <c r="I111" s="7" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡最大篝火夜之一；有音乐舞台和游乐场；没有售票数据</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="L111" s="5" t="inlineStr">
+        <is>
+          <t>离 Huddersfield 约 10 公里，比市内的活动规模大</t>
+        </is>
+      </c>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O111" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="58" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>university of york student hub</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>待制作：university of york student hub.png</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>🔍 Event Radar (UK) — what's worth doing this month.
+This month: YORK 👇
+🎄 York Christmas Market, Parliament Street, York — one of the UK's best festive markets (closed Tuesdays), from 12 Nov.
+🌿 RHS Glow at Harlow Carr, Harrogate — a garden lit up for its 10th year, from 26 Nov.</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>York Christmas Market（St Nicholas Fair）</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Parliament Street &amp; St Sampson's Square, York YO1</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>12 Nov – 21 Dec 2026，10:30–19:00（周二不开，今年试行）</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>本地生活类(集市) + 一日游</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J112" s="5" t="inlineStr">
+        <is>
+          <t>Make It York 官方公布 2026 年日期和营业时间；英国最有名的圣诞市集之一</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>https://www.makeityork.com/news/2026/08/york-christmas-market-2026-dates-announced/ ; https://visityork.org/christmas/york-christmas-market</t>
+        </is>
+      </c>
+      <c r="L112" s="5" t="inlineStr">
+        <is>
+          <t>免费；⚠️周二不开；古城加圣诞市集，很适合一日游</t>
+        </is>
+      </c>
+      <c r="M112" s="5" t="inlineStr">
+        <is>
+          <t>Day Trip Buddies</t>
+        </is>
+      </c>
+      <c r="N112" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O112" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="58" customHeight="1">
+      <c r="A113" s="2" t="n"/>
+      <c r="B113" s="3" t="n"/>
+      <c r="C113" s="4" t="n"/>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
           <t>RHS Glow：Harlow Carr 灯光花园（10 周年）</t>
         </is>
       </c>
-      <c r="E110" s="2" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>RHS Garden Harlow Carr, Crag Lane, Harrogate HG3 1QB</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="F113" s="2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="G110" s="5" t="inlineStr">
+      <c r="G113" s="5" t="inlineStr">
         <is>
           <t>26 Nov – 30 Dec 2026（指定日期开放）</t>
         </is>
       </c>
-      <c r="H110" s="5" t="inlineStr">
+      <c r="H113" s="5" t="inlineStr">
         <is>
           <t>兴趣类(园艺) + 灯光步道</t>
         </is>
       </c>
-      <c r="I110" s="6" t="inlineStr">
+      <c r="I113" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J110" s="5" t="inlineStr">
+      <c r="J113" s="5" t="inlineStr">
         <is>
           <t>RHS 官方页面公布；Harlow Carr 场办到第 10 年，今年新增 off-peak 票</t>
         </is>
       </c>
-      <c r="K110" s="5" t="inlineStr">
+      <c r="K113" s="5" t="inlineStr">
         <is>
           <t>https://www.rhs.org.uk/gardens/articles/glow-illuminations</t>
         </is>
       </c>
-      <c r="L110" s="5" t="inlineStr">
+      <c r="L113" s="5" t="inlineStr">
         <is>
           <t>离 York、Leeds 都约 35 公里；分时段预约</t>
         </is>
       </c>
-      <c r="M110" s="5" t="inlineStr">
+      <c r="M113" s="5" t="inlineStr">
         <is>
           <t>Green Thumb Circle</t>
         </is>
       </c>
-      <c r="N110" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O110" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="60" customHeight="1">
-      <c r="A111" s="2" t="inlineStr">
+      <c r="N113" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O113" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="60" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>Hull Uni Student Hub</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B114" s="3" t="inlineStr">
         <is>
           <t>待制作：Hull Uni Student Hub.png</t>
         </is>
       </c>
-      <c r="C111" s="4" t="inlineStr">
+      <c r="C114" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: HULL 👇
 🎸 Squeeze with Billy Bragg, Connexin Live, Hull — two British songwriting legends, 19 Nov.</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D114" s="2" t="inlineStr">
         <is>
           <t>Squeeze（嘉宾 Billy Bragg）巡演 赫尔站</t>
         </is>
       </c>
-      <c r="E111" s="2" t="inlineStr">
+      <c r="E114" s="2" t="inlineStr">
         <is>
           <t>Connexin Live（原 Bonus Arena）, Hull city centre</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr">
+      <c r="F114" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G111" s="5" t="inlineStr">
+      <c r="G114" s="5" t="inlineStr">
         <is>
           <t>19 Nov 2026（周四）</t>
         </is>
       </c>
-      <c r="H111" s="5" t="inlineStr">
+      <c r="H114" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(Live Music)</t>
         </is>
       </c>
-      <c r="I111" s="6" t="inlineStr">
+      <c r="I114" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J111" s="5" t="inlineStr">
+      <c r="J114" s="5" t="inlineStr">
         <is>
           <t>场馆官网列出；同一巡演 20 Nov 在 Leeds arena，日程对得上；场馆页面信息可能更新不及时</t>
         </is>
       </c>
-      <c r="K111" s="5" t="inlineStr">
+      <c r="K114" s="5" t="inlineStr">
         <is>
           <t>https://connexinlivehull.com/whats-on/</t>
         </is>
       </c>
-      <c r="L111" s="5" t="inlineStr">
+      <c r="L114" s="5" t="inlineStr">
         <is>
           <t>Hull 本月少见的大牌演出；推之前确认一下票务页</t>
         </is>
       </c>
-      <c r="M111" s="5" t="inlineStr">
+      <c r="M114" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N111" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O111" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="58" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
+      <c r="N114" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O114" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="58" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B115" s="3" t="inlineStr">
         <is>
           <t>待制作：Newcastle university.png</t>
         </is>
       </c>
-      <c r="C112" s="4" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: NEWCASTLE 👇
@@ -8399,249 +8597,54 @@
 💡 Northern Lights Newcastle, Leazes Park — 14 new light installations next to campus, from 20 Nov.</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D115" s="2" t="inlineStr">
         <is>
           <t>Newcastle Christmas Market + Christmas Village</t>
         </is>
       </c>
-      <c r="E112" s="2" t="inlineStr">
+      <c r="E115" s="2" t="inlineStr">
         <is>
           <t>Grey Street / Grainger Street / Monument / Nelson Street（市集）；Old Eldon Square（Christmas Village）, Newcastle</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr">
+      <c r="F115" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G112" s="5" t="inlineStr">
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>19 Nov – 23 Dec 2026</t>
         </is>
       </c>
-      <c r="H112" s="5" t="inlineStr">
+      <c r="H115" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市)</t>
         </is>
       </c>
-      <c r="I112" s="8" t="inlineStr">
+      <c r="I115" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J112" s="5" t="inlineStr">
+      <c r="J115" s="5" t="inlineStr">
         <is>
           <t>Newcastle 市议会公布；70 多个摊位，86% 是本地商家</t>
         </is>
       </c>
-      <c r="K112" s="5" t="inlineStr">
+      <c r="K115" s="5" t="inlineStr">
         <is>
           <t>https://new.newcastle.gov.uk/news/2026/newcastles-christmas-set-biggest-year-yet-after-festive-market-success</t>
         </is>
       </c>
-      <c r="L112" s="5" t="inlineStr">
+      <c r="L115" s="5" t="inlineStr">
         <is>
           <t>免费；Northumbria 和 Newcastle 大学都在市中心旁边</t>
         </is>
       </c>
-      <c r="M112" s="5" t="inlineStr">
+      <c r="M115" s="5" t="inlineStr">
         <is>
           <t>Durham university</t>
-        </is>
-      </c>
-      <c r="N112" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O112" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="58" customHeight="1">
-      <c r="A113" s="2" t="n"/>
-      <c r="B113" s="3" t="n"/>
-      <c r="C113" s="4" t="n"/>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
-        </is>
-      </c>
-      <c r="H113" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(烟花/赛马)</t>
-        </is>
-      </c>
-      <c r="I113" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J113" s="5" t="inlineStr">
-        <is>
-          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
-        </is>
-      </c>
-      <c r="K113" s="5" t="inlineStr">
-        <is>
-          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
-        </is>
-      </c>
-      <c r="L113" s="5" t="inlineStr">
-        <is>
-          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
-        </is>
-      </c>
-      <c r="M113" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N113" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O113" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="71.5" customHeight="1">
-      <c r="A114" s="2" t="n"/>
-      <c r="B114" s="3" t="n"/>
-      <c r="C114" s="4" t="n"/>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>Reverend and The Makers 演唱会</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>14 Nov 2026（周六）19:00 开门</t>
-        </is>
-      </c>
-      <c r="H114" s="5" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
-        </is>
-      </c>
-      <c r="I114" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J114" s="5" t="inlineStr">
-        <is>
-          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
-        </is>
-      </c>
-      <c r="K114" s="5" t="inlineStr">
-        <is>
-          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
-        </is>
-      </c>
-      <c r="L114" s="5" t="inlineStr">
-        <is>
-          <t>就在 Northumbria 学生会里，在校生走路就到</t>
-        </is>
-      </c>
-      <c r="M114" s="5" t="inlineStr">
-        <is>
-          <t>Live Music Crew</t>
-        </is>
-      </c>
-      <c r="N114" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O114" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="71.5" customHeight="1">
-      <c r="A115" s="2" t="n"/>
-      <c r="B115" s="3" t="n"/>
-      <c r="C115" s="4" t="n"/>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>Newcastle 圣诞亮灯仪式</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>Grey's Monument, Grey Street, Newcastle upon Tyne NE1</t>
-        </is>
-      </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>venue_only</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>12 Nov 2026（周四）约 18:00–19:00</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr">
-        <is>
-          <t>本地生活类(节庆)</t>
-        </is>
-      </c>
-      <c r="I115" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J115" s="5" t="inlineStr">
-        <is>
-          <t>Newcastle 市议会 2026 年新闻稿公布日期；免费；具体时间参考往年</t>
-        </is>
-      </c>
-      <c r="K115" s="5" t="inlineStr">
-        <is>
-          <t>https://new.newcastle.gov.uk/news/2026/newcastles-christmas-set-biggest-year-yet-after-festive-market-success ; https://newcastlegateshead.com/events/newcastle-christmas-light-switch-on</t>
-        </is>
-      </c>
-      <c r="L115" s="5" t="inlineStr">
-        <is>
-          <t>免费，市中心，下课后顺路</t>
-        </is>
-      </c>
-      <c r="M115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
       <c r="N115" s="5" t="inlineStr">
@@ -8661,156 +8664,351 @@
       <c r="C116" s="4" t="n"/>
       <c r="D116" s="2" t="inlineStr">
         <is>
+          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/赛马)</t>
+        </is>
+      </c>
+      <c r="I116" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J116" s="5" t="inlineStr">
+        <is>
+          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
+        </is>
+      </c>
+      <c r="K116" s="5" t="inlineStr">
+        <is>
+          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
+        </is>
+      </c>
+      <c r="L116" s="5" t="inlineStr">
+        <is>
+          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
+        </is>
+      </c>
+      <c r="M116" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N116" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O116" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="71.5" customHeight="1">
+      <c r="A117" s="2" t="n"/>
+      <c r="B117" s="3" t="n"/>
+      <c r="C117" s="4" t="n"/>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Reverend and The Makers 演唱会</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>14 Nov 2026（周六）19:00 开门</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+        </is>
+      </c>
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="inlineStr">
+        <is>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+        </is>
+      </c>
+      <c r="L117" s="5" t="inlineStr">
+        <is>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+        </is>
+      </c>
+      <c r="M117" s="5" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="N117" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O117" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="71.5" customHeight="1">
+      <c r="A118" s="2" t="n"/>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="4" t="n"/>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle 圣诞亮灯仪式</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>Grey's Monument, Grey Street, Newcastle upon Tyne NE1</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>12 Nov 2026（周四）约 18:00–19:00</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>本地生活类(节庆)</t>
+        </is>
+      </c>
+      <c r="I118" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J118" s="5" t="inlineStr">
+        <is>
+          <t>Newcastle 市议会 2026 年新闻稿公布日期；免费；具体时间参考往年</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>https://new.newcastle.gov.uk/news/2026/newcastles-christmas-set-biggest-year-yet-after-festive-market-success ; https://newcastlegateshead.com/events/newcastle-christmas-light-switch-on</t>
+        </is>
+      </c>
+      <c r="L118" s="5" t="inlineStr">
+        <is>
+          <t>免费，市中心，下课后顺路</t>
+        </is>
+      </c>
+      <c r="M118" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N118" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O118" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="58" customHeight="1">
+      <c r="A119" s="2" t="n"/>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="4" t="n"/>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
           <t>Northern Lights Newcastle 灯光步道</t>
         </is>
       </c>
-      <c r="E116" s="2" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>Leazes Park, Newcastle upon Tyne</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
+      <c r="F119" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G116" s="5" t="inlineStr">
+      <c r="G119" s="5" t="inlineStr">
         <is>
           <t>20 Nov – 31 Dec 2026（23、24、25、30 Nov 不开），约 16:15–20:30</t>
         </is>
       </c>
-      <c r="H116" s="5" t="inlineStr">
+      <c r="H119" s="5" t="inlineStr">
         <is>
           <t>本地生活类(灯光步道)</t>
         </is>
       </c>
-      <c r="I116" s="6" t="inlineStr">
+      <c r="I119" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J116" s="5" t="inlineStr">
+      <c r="J119" s="5" t="inlineStr">
         <is>
           <t>Newcastle 市议会活动页列出；今年 14 个新装置</t>
         </is>
       </c>
-      <c r="K116" s="5" t="inlineStr">
+      <c r="K119" s="5" t="inlineStr">
         <is>
           <t>https://new.newcastle.gov.uk/events/northern-lights-2026 ; https://northernlightsnewcastle.com/</t>
         </is>
       </c>
-      <c r="L116" s="5" t="inlineStr">
+      <c r="L119" s="5" t="inlineStr">
         <is>
           <t>Leazes Park 就在 Newcastle 大学旁边</t>
         </is>
       </c>
-      <c r="M116" s="5" t="inlineStr">
+      <c r="M119" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N116" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O116" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="60" customHeight="1">
-      <c r="A117" s="2" t="inlineStr">
+      <c r="N119" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O119" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="60" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>Durham university</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B120" s="3" t="inlineStr">
         <is>
           <t>待制作：Durham university.png</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: DURHAM &amp; NEWCASTLE 👇
 🎄 Newcastle Christmas Market, 15 min by train from Durham — 70+ mostly local traders, from 19 Nov.</t>
         </is>
       </c>
-      <c r="D117" s="2" t="inlineStr">
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>Newcastle Christmas Market + Christmas Village</t>
         </is>
       </c>
-      <c r="E117" s="2" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>Grey Street / Grainger Street / Monument / Nelson Street（市集）；Old Eldon Square（Christmas Village）, Newcastle</t>
         </is>
       </c>
-      <c r="F117" s="2" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G117" s="5" t="inlineStr">
+      <c r="G120" s="5" t="inlineStr">
         <is>
           <t>19 Nov – 23 Dec 2026</t>
         </is>
       </c>
-      <c r="H117" s="5" t="inlineStr">
+      <c r="H120" s="5" t="inlineStr">
         <is>
           <t>本地生活类(集市)</t>
         </is>
       </c>
-      <c r="I117" s="8" t="inlineStr">
+      <c r="I120" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J117" s="5" t="inlineStr">
+      <c r="J120" s="5" t="inlineStr">
         <is>
           <t>Newcastle 市议会公布；70 多个摊位，86% 是本地商家</t>
         </is>
       </c>
-      <c r="K117" s="5" t="inlineStr">
+      <c r="K120" s="5" t="inlineStr">
         <is>
           <t>https://new.newcastle.gov.uk/news/2026/newcastles-christmas-set-biggest-year-yet-after-festive-market-success</t>
         </is>
       </c>
-      <c r="L117" s="5" t="inlineStr">
+      <c r="L120" s="5" t="inlineStr">
         <is>
           <t>免费；Northumbria 和 Newcastle 大学都在市中心旁边</t>
         </is>
       </c>
-      <c r="M117" s="5" t="inlineStr">
+      <c r="M120" s="5" t="inlineStr">
         <is>
           <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
         </is>
       </c>
-      <c r="N117" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O117" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="58" customHeight="1">
-      <c r="A118" s="2" t="inlineStr">
+      <c r="N120" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O120" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="58" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
         <is>
           <t>University of Cardiff / Cardiff Metropolitan University</t>
         </is>
       </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B121" s="3" t="inlineStr">
         <is>
           <t>待制作：University of Cardiff.png</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: CARDIFF 👇
@@ -8822,244 +9020,49 @@
 💡 Christmas at Bute Park, Cardiff — a reimagined light trail next to the castle, from 19 Nov.</t>
         </is>
       </c>
-      <c r="D118" s="2" t="inlineStr">
+      <c r="D121" s="2" t="inlineStr">
         <is>
           <t>Cardiff's Winter Wonderland 2026（冰场 / 摩天轮 / 冰壶）</t>
         </is>
       </c>
-      <c r="E118" s="2" t="inlineStr">
+      <c r="E121" s="2" t="inlineStr">
         <is>
           <t>Cardiff Castle, Castle Street, Cardiff CF10 3RB &amp; City Hall Lawn</t>
         </is>
       </c>
-      <c r="F118" s="2" t="inlineStr">
+      <c r="F121" s="2" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="G118" s="5" t="inlineStr">
+      <c r="G121" s="5" t="inlineStr">
         <is>
           <t>12 Nov 2026 – 3 Jan 2027（窗口内为 12–30 Nov）</t>
         </is>
       </c>
-      <c r="H118" s="5" t="inlineStr">
+      <c r="H121" s="5" t="inlineStr">
         <is>
           <t>年轻人娱乐(滑冰/游乐)</t>
         </is>
       </c>
-      <c r="I118" s="8" t="inlineStr">
+      <c r="I121" s="8" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J118" s="5" t="inlineStr">
+      <c r="J121" s="5" t="inlineStr">
         <is>
           <t>Visit Cardiff 官方收录，年年举办；Nation.Cymru、Wales247 报道了 2026 年日期</t>
         </is>
       </c>
-      <c r="K118" s="5" t="inlineStr">
+      <c r="K121" s="5" t="inlineStr">
         <is>
           <t>https://www.visitcardiff.com/christmas/cardiffs-winter-wonderland/ ; https://www.wales247.co.uk/cardiff-confirms-christmas-lights-date-and-festive-attractions-for-2026</t>
         </is>
       </c>
-      <c r="L118" s="5" t="inlineStr">
+      <c r="L121" s="5" t="inlineStr">
         <is>
           <t>城堡里的露天冰场很出片；今年新增冰壶体验</t>
-        </is>
-      </c>
-      <c r="M118" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N118" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O118" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="71.5" customHeight="1">
-      <c r="A119" s="2" t="n"/>
-      <c r="B119" s="3" t="n"/>
-      <c r="C119" s="4" t="n"/>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>威尔士 vs 日本（Nations Championship 橄榄球）</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G119" s="5" t="inlineStr">
-        <is>
-          <t>7 Nov 2026（周六）16:40 开球</t>
-        </is>
-      </c>
-      <c r="H119" s="5" t="inlineStr">
-        <is>
-          <t>运动户外(观赛)</t>
-        </is>
-      </c>
-      <c r="I119" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J119" s="5" t="inlineStr">
-        <is>
-          <t>WRU 官方公布；球场官网有单场售票页</t>
-        </is>
-      </c>
-      <c r="K119" s="5" t="inlineStr">
-        <is>
-          <t>https://www.wru.wales/2026/03/dates-confirmed-for-wales-home-nations-championship-fixtures ; https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-japan/</t>
-        </is>
-      </c>
-      <c r="L119" s="5" t="inlineStr">
-        <is>
-          <t>市中心球场，比赛日全城都是气氛；对日本这场的票通常比对新西兰便宜</t>
-        </is>
-      </c>
-      <c r="M119" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N119" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O119" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="58" customHeight="1">
-      <c r="A120" s="2" t="n"/>
-      <c r="B120" s="3" t="n"/>
-      <c r="C120" s="4" t="n"/>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>威尔士 vs 新西兰（Nations Championship 橄榄球）</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G120" s="5" t="inlineStr">
-        <is>
-          <t>14 Nov 2026（周六）</t>
-        </is>
-      </c>
-      <c r="H120" s="5" t="inlineStr">
-        <is>
-          <t>运动户外(观赛)</t>
-        </is>
-      </c>
-      <c r="I120" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J120" s="5" t="inlineStr">
-        <is>
-          <t>WRU 官方公布；对全黑队是秋季重头戏</t>
-        </is>
-      </c>
-      <c r="K120" s="5" t="inlineStr">
-        <is>
-          <t>https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-new-zealand/</t>
-        </is>
-      </c>
-      <c r="L120" s="5" t="inlineStr">
-        <is>
-          <t>⚠️对全黑队的票最贵；买不到票也可以去市中心酒吧看直播</t>
-        </is>
-      </c>
-      <c r="M120" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N120" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O120" s="5" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="71.5" customHeight="1">
-      <c r="A121" s="2" t="n"/>
-      <c r="B121" s="3" t="n"/>
-      <c r="C121" s="4" t="n"/>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>威尔士 vs 澳大利亚（Nations Championship 橄榄球）</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G121" s="5" t="inlineStr">
-        <is>
-          <t>21 Nov 2026（周六）20:10 开球</t>
-        </is>
-      </c>
-      <c r="H121" s="5" t="inlineStr">
-        <is>
-          <t>运动户外(观赛)</t>
-        </is>
-      </c>
-      <c r="I121" s="8" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J121" s="5" t="inlineStr">
-        <is>
-          <t>Visit Wales、World Rugby 都列出；威尔士 11 月三场主场赛的最后一场</t>
-        </is>
-      </c>
-      <c r="K121" s="5" t="inlineStr">
-        <is>
-          <t>https://www.visitwales.com/event/sporting-event/nations-championship-2026-wales-v-australia-620271 ; https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-australia/</t>
-        </is>
-      </c>
-      <c r="L121" s="5" t="inlineStr">
-        <is>
-          <t>晚场比赛，市中心气氛最好；同一天还有 Bloc Party &amp; Interpol 演唱会，可二选一</t>
         </is>
       </c>
       <c r="M121" s="5" t="inlineStr">
@@ -9084,47 +9087,47 @@
       <c r="C122" s="4" t="n"/>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Bloc Party &amp; Interpol 联合巡演 卡迪夫站</t>
+          <t>威尔士 vs 日本（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Utilita Arena Cardiff, Mary Ann Street, Cardiff</t>
+          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>21 Nov 2026（周六）</t>
+          <t>7 Nov 2026（周六）16:40 开球</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
-        </is>
-      </c>
-      <c r="I122" s="6" t="inlineStr">
-        <is>
-          <t>中热度</t>
+          <t>运动户外(观赛)</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
         </is>
       </c>
       <c r="J122" s="5" t="inlineStr">
         <is>
-          <t>巡演日程（Songkick 报道）里伯明翰站之后的下一站；具体开场时间看票务页</t>
+          <t>WRU 官方公布；球场官网有单场售票页</t>
         </is>
       </c>
       <c r="K122" s="5" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/concerts/42867381-bloc-party-at-utilita-arena-birmingham ; https://www.thelineofbestfit.com/news/bloc-party-and-interpol-announce-2026-uk-eu-co-headline-tour</t>
+          <t>https://www.wru.wales/2026/03/dates-confirmed-for-wales-home-nations-championship-fixtures ; https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-japan/</t>
         </is>
       </c>
       <c r="L122" s="5" t="inlineStr">
         <is>
-          <t>和威尔士 vs 澳大利亚同一天，二选一</t>
+          <t>市中心球场，比赛日全城都是气氛；对日本这场的票通常比对新西兰便宜</t>
         </is>
       </c>
       <c r="M122" s="5" t="inlineStr">
@@ -9149,162 +9152,357 @@
       <c r="C123" s="4" t="n"/>
       <c r="D123" s="2" t="inlineStr">
         <is>
+          <t>威尔士 vs 新西兰（Nations Championship 橄榄球）</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>14 Nov 2026（周六）</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>运动户外(观赛)</t>
+        </is>
+      </c>
+      <c r="I123" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J123" s="5" t="inlineStr">
+        <is>
+          <t>WRU 官方公布；对全黑队是秋季重头戏</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-new-zealand/</t>
+        </is>
+      </c>
+      <c r="L123" s="5" t="inlineStr">
+        <is>
+          <t>⚠️对全黑队的票最贵；买不到票也可以去市中心酒吧看直播</t>
+        </is>
+      </c>
+      <c r="M123" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N123" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O123" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="71.5" customHeight="1">
+      <c r="A124" s="2" t="n"/>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="4" t="n"/>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>威尔士 vs 澳大利亚（Nations Championship 橄榄球）</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Principality Stadium, Westgate Street, Cardiff CF10 1NS</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>21 Nov 2026（周六）20:10 开球</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>运动户外(观赛)</t>
+        </is>
+      </c>
+      <c r="I124" s="8" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J124" s="5" t="inlineStr">
+        <is>
+          <t>Visit Wales、World Rugby 都列出；威尔士 11 月三场主场赛的最后一场</t>
+        </is>
+      </c>
+      <c r="K124" s="5" t="inlineStr">
+        <is>
+          <t>https://www.visitwales.com/event/sporting-event/nations-championship-2026-wales-v-australia-620271 ; https://www.principalitystadium.wales/event/nations-championship-2026-wales-v-australia/</t>
+        </is>
+      </c>
+      <c r="L124" s="5" t="inlineStr">
+        <is>
+          <t>晚场比赛，市中心气氛最好；同一天还有 Bloc Party &amp; Interpol 演唱会，可二选一</t>
+        </is>
+      </c>
+      <c r="M124" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N124" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O124" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="71.5" customHeight="1">
+      <c r="A125" s="2" t="n"/>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="4" t="n"/>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Bloc Party &amp; Interpol 联合巡演 卡迪夫站</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>Utilita Arena Cardiff, Mary Ann Street, Cardiff</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>21 Nov 2026（周六）</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+        </is>
+      </c>
+      <c r="I125" s="6" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J125" s="5" t="inlineStr">
+        <is>
+          <t>巡演日程（Songkick 报道）里伯明翰站之后的下一站；具体开场时间看票务页</t>
+        </is>
+      </c>
+      <c r="K125" s="5" t="inlineStr">
+        <is>
+          <t>https://www.songkick.com/concerts/42867381-bloc-party-at-utilita-arena-birmingham ; https://www.thelineofbestfit.com/news/bloc-party-and-interpol-announce-2026-uk-eu-co-headline-tour</t>
+        </is>
+      </c>
+      <c r="L125" s="5" t="inlineStr">
+        <is>
+          <t>和威尔士 vs 澳大利亚同一天，二选一</t>
+        </is>
+      </c>
+      <c r="M125" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N125" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O125" s="5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="58" customHeight="1">
+      <c r="A126" s="2" t="n"/>
+      <c r="B126" s="3" t="n"/>
+      <c r="C126" s="4" t="n"/>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
           <t>Christmas at Bute Park 灯光步道</t>
         </is>
       </c>
-      <c r="E123" s="2" t="inlineStr">
+      <c r="E126" s="2" t="inlineStr">
         <is>
           <t>Bute Park（Cardiff Castle 旁）, Cardiff</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr">
+      <c r="F126" s="2" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G123" s="5" t="inlineStr">
+      <c r="G126" s="5" t="inlineStr">
         <is>
           <t>19 Nov – 31 Dec 2026，16:15 起入场</t>
         </is>
       </c>
-      <c r="H123" s="5" t="inlineStr">
+      <c r="H126" s="5" t="inlineStr">
         <is>
           <t>本地生活类(灯光步道)</t>
         </is>
       </c>
-      <c r="I123" s="6" t="inlineStr">
+      <c r="I126" s="6" t="inlineStr">
         <is>
           <t>中热度</t>
         </is>
       </c>
-      <c r="J123" s="5" t="inlineStr">
+      <c r="J126" s="5" t="inlineStr">
         <is>
           <t>Visit Cardiff 官方收录；今年路线重新设计；See Tickets 正规售票</t>
         </is>
       </c>
-      <c r="K123" s="5" t="inlineStr">
+      <c r="K126" s="5" t="inlineStr">
         <is>
           <t>https://www.visitcardiff.com/events/christmas-lights-bute-park/ ; https://christmasatbute.seetickets.com/timeslot/christmas-at-bute-park/</t>
         </is>
       </c>
-      <c r="L123" s="5" t="inlineStr">
+      <c r="L126" s="5" t="inlineStr">
         <is>
           <t>peak 票 £17.25 起、off-peak £13.75 起；离 Cardiff 大学主校区很近</t>
         </is>
       </c>
-      <c r="M123" s="5" t="inlineStr">
+      <c r="M126" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N123" s="5" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O123" s="5" t="inlineStr">
+      <c r="N126" s="5" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O126" s="5" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O123"/>
+  <autoFilter ref="A1:O126"/>
   <mergeCells count="96">
     <mergeCell ref="C30:C31"/>
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="B82:B86"/>
     <mergeCell ref="C32:C34"/>
-    <mergeCell ref="C98:C103"/>
-    <mergeCell ref="C93:C94"/>
+    <mergeCell ref="B109:B111"/>
     <mergeCell ref="B76:B80"/>
     <mergeCell ref="C22:C29"/>
-    <mergeCell ref="C86:C87"/>
-    <mergeCell ref="B118:B123"/>
-    <mergeCell ref="C88:C92"/>
-    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="A82:A86"/>
+    <mergeCell ref="A121:A126"/>
     <mergeCell ref="A10:A15"/>
     <mergeCell ref="A55:A59"/>
     <mergeCell ref="A35:A38"/>
+    <mergeCell ref="C115:C119"/>
     <mergeCell ref="C55:C59"/>
+    <mergeCell ref="C98:C99"/>
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B93:B94"/>
     <mergeCell ref="A70:A71"/>
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="A32:A34"/>
+    <mergeCell ref="C112:C113"/>
     <mergeCell ref="C35:C38"/>
-    <mergeCell ref="A106:A108"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="C109:C110"/>
+    <mergeCell ref="A87:A88"/>
     <mergeCell ref="A74:A75"/>
-    <mergeCell ref="A112:A116"/>
+    <mergeCell ref="B121:B126"/>
+    <mergeCell ref="A89:A90"/>
     <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="C95:C96"/>
+    <mergeCell ref="B115:B119"/>
     <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B91:B95"/>
     <mergeCell ref="C17:C18"/>
     <mergeCell ref="A60:A62"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="B95:B96"/>
     <mergeCell ref="A68:A69"/>
     <mergeCell ref="C63:C67"/>
     <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C87:C88"/>
     <mergeCell ref="C74:C75"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="C68:C69"/>
+    <mergeCell ref="A107:A108"/>
+    <mergeCell ref="C107:C108"/>
+    <mergeCell ref="C101:C106"/>
     <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A84:A85"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="A109:A111"/>
     <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B82:B83"/>
     <mergeCell ref="B22:B29"/>
     <mergeCell ref="C44:C45"/>
-    <mergeCell ref="C84:C85"/>
     <mergeCell ref="B63:B67"/>
-    <mergeCell ref="B98:B103"/>
+    <mergeCell ref="C82:C86"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="B107:B108"/>
     <mergeCell ref="B68:B69"/>
-    <mergeCell ref="A118:A123"/>
-    <mergeCell ref="C118:C123"/>
     <mergeCell ref="C70:C71"/>
-    <mergeCell ref="A104:A105"/>
-    <mergeCell ref="A88:A92"/>
     <mergeCell ref="B10:B15"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C39:C40"/>
+    <mergeCell ref="A112:A113"/>
     <mergeCell ref="B5:B8"/>
     <mergeCell ref="A48:A54"/>
-    <mergeCell ref="A93:A94"/>
     <mergeCell ref="B19:B21"/>
+    <mergeCell ref="A98:A99"/>
     <mergeCell ref="B72:B73"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B35:B38"/>
-    <mergeCell ref="B109:B110"/>
-    <mergeCell ref="A98:A103"/>
     <mergeCell ref="C76:C80"/>
+    <mergeCell ref="B96:B97"/>
     <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C104:C105"/>
+    <mergeCell ref="C89:C90"/>
+    <mergeCell ref="C91:C95"/>
     <mergeCell ref="B55:B59"/>
     <mergeCell ref="A63:A67"/>
+    <mergeCell ref="A115:A119"/>
     <mergeCell ref="B39:B40"/>
+    <mergeCell ref="A91:A95"/>
     <mergeCell ref="C48:C54"/>
-    <mergeCell ref="A86:A87"/>
     <mergeCell ref="A19:A21"/>
+    <mergeCell ref="C121:C126"/>
     <mergeCell ref="C10:C15"/>
     <mergeCell ref="C19:C21"/>
-    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="B101:B106"/>
     <mergeCell ref="B32:B34"/>
-    <mergeCell ref="B106:B108"/>
+    <mergeCell ref="B87:B88"/>
+    <mergeCell ref="A101:A106"/>
     <mergeCell ref="B74:B75"/>
-    <mergeCell ref="A109:A110"/>
     <mergeCell ref="A72:A73"/>
     <mergeCell ref="C72:C73"/>
+    <mergeCell ref="A96:A97"/>
     <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="C96:C97"/>
     <mergeCell ref="A44:A45"/>
+    <mergeCell ref="C109:C111"/>
     <mergeCell ref="B60:B62"/>
-    <mergeCell ref="C112:C116"/>
-    <mergeCell ref="A82:A83"/>
     <mergeCell ref="A22:A29"/>
     <mergeCell ref="A30:A31"/>
   </mergeCells>
@@ -10547,11 +10745,11 @@
         </is>
       </c>
       <c r="D48" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>未达 3–5 条</t>
+          <t>和 Warwick 合并发布；Coventry 2026 年圣诞市集和摩天轮还没公布（2025 年是 21 Nov 开），学生会活动页没写年份，都没收录</t>
         </is>
       </c>
     </row>
@@ -10572,11 +10770,11 @@
         </is>
       </c>
       <c r="D49" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>未达 3–5 条</t>
+          <t>和 Coventry 合并发布；Warwick Arts Centre 的喜剧场就在校园里</t>
         </is>
       </c>
     </row>

</xml_diff>